<commit_message>
Streamline multi-project reconciliation with explicit original currency and base amount review
</commit_message>
<xml_diff>
--- a/examples/项目A往来.xlsx
+++ b/examples/项目A往来.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="往来明细" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="往来辅助明细账" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>本方项目</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -429,97 +429,216 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>记账日期</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>原币币种</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>原币借方发生额</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>原币贷方发生额</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>本币币种</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>本币借方发生额</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>本币贷方发生额</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>参考号</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>摘要</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>借方金额</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>贷方金额</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>参考号</t>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>科目编码</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>科目名称</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>项目A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>项目B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>项目B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>7300</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>拨付B项目</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>AB1</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1221</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>其他应收款</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>项目A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>项目C</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>2026-01-06</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>项目C</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>500</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>3600</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>拨付C项目</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>500</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>AC1</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1221</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>其他应收款</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>项目A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>项目D</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>2026-01-07</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>项目D</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>对方账簿未提供</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>80</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>AD1</t>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>576</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>未提供对方账簿</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1221</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>其他应收款</t>
         </is>
       </c>
     </row>

</xml_diff>